<commit_message>
feat: comprehensive Telegram and scheduler improvements
Catch-up Logic Redesign:
- Run ALL missed slots instead of just one on late start
- If scheduler starts at 9:30, now runs 09:00, 09:08, 09:15, 09:30 catch-ups
- Each catch-up message has proper slot config (no more single generic catch-up)
- Pass scheduled_slots to run_loop for accurate missed slot detection

Telegram Formatting Enhancements:
- Add HTML table formatting for FII/DII Buy/Sell/Net (better alignment)
- Add table formatting for Highest Value Traded (cleaner layout)
- Fix duplicate stocks in Highest Value Traded (deduplicate by symbol)
- Add negative operator for Sell amounts (Buy +₹X | Sell -₹Y)
- Add timestamp to 'Changes vs Last Check' and 'Since Last Check' sections
- New helper: _make_table() for ASCII table generation with alignment
- New helper: _format_prev_time() for consistent timestamp formatting

Fixes:
- Add List type import in scheduler.py
- Return scheduled_times from setup_schedule() for catch-up logic
</commit_message>
<xml_diff>
--- a/data/excel/market_tracker.xlsx
+++ b/data/excel/market_tracker.xlsx
@@ -1098,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19" customWidth="1" style="18" min="1" max="1"/>
@@ -1472,6 +1472,135 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>02-Mar-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>12737.34</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>16032.98</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>-3295.64</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>21110.66</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>12516.79</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>8593.870000000001</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>5298.230000000001</v>
+      </c>
+      <c r="J9" s="22" t="inlineStr">
+        <is>
+          <t>DII Defensive</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
+        <is>
+          <t>FII selling, DII buying — DII supporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>02-Mar-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>12737.34</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>16032.98</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>-3295.64</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>21110.66</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <v>12516.79</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>8593.870000000001</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>5298.230000000001</v>
+      </c>
+      <c r="J10" s="22" t="inlineStr">
+        <is>
+          <t>DII Defensive</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
+        <is>
+          <t>FII selling, DII buying — DII supporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>02-Mar-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>12737.34</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>16032.98</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>-3295.64</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>21110.66</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>12516.79</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>8593.870000000001</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>5298.230000000001</v>
+      </c>
+      <c r="J11" s="22" t="inlineStr">
+        <is>
+          <t>DII Defensive</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="inlineStr">
+        <is>
+          <t>FII selling, DII buying — DII supporting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1484,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" ht="27.6" customHeight="1" s="18">
@@ -7803,6 +7932,2703 @@
         </is>
       </c>
       <c r="K148" s="22" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B149" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C149" s="22" t="n">
+        <v>24865.7</v>
+      </c>
+      <c r="D149" s="22" t="n">
+        <v>-312.95</v>
+      </c>
+      <c r="E149" s="23" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="F149" s="22" t="n">
+        <v>24659.25</v>
+      </c>
+      <c r="G149" s="22" t="n">
+        <v>24989.35</v>
+      </c>
+      <c r="H149" s="22" t="n">
+        <v>24603.5</v>
+      </c>
+      <c r="I149" s="22" t="n">
+        <v>25178.65</v>
+      </c>
+      <c r="J149" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K149" s="22" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B150" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY NEXT 50</t>
+        </is>
+      </c>
+      <c r="C150" s="22" t="n">
+        <v>68650.25</v>
+      </c>
+      <c r="D150" s="22" t="n">
+        <v>-1060.65</v>
+      </c>
+      <c r="E150" s="23" t="n">
+        <v>-1.52</v>
+      </c>
+      <c r="F150" s="22" t="n">
+        <v>67393.3</v>
+      </c>
+      <c r="G150" s="22" t="n">
+        <v>69144.45</v>
+      </c>
+      <c r="H150" s="22" t="n">
+        <v>67352.55</v>
+      </c>
+      <c r="I150" s="22" t="n">
+        <v>69710.89999999999</v>
+      </c>
+      <c r="J150" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K150" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B151" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY BANK</t>
+        </is>
+      </c>
+      <c r="C151" s="22" t="n">
+        <v>59839.65</v>
+      </c>
+      <c r="D151" s="22" t="n">
+        <v>-689.35</v>
+      </c>
+      <c r="E151" s="23" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="F151" s="22" t="n">
+        <v>59204.3</v>
+      </c>
+      <c r="G151" s="22" t="n">
+        <v>60177.5</v>
+      </c>
+      <c r="H151" s="22" t="n">
+        <v>59148</v>
+      </c>
+      <c r="I151" s="22" t="n">
+        <v>60529</v>
+      </c>
+      <c r="J151" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K151" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B152" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FINANCIAL SERVICES</t>
+        </is>
+      </c>
+      <c r="C152" s="22" t="n">
+        <v>27564.1</v>
+      </c>
+      <c r="D152" s="22" t="n">
+        <v>-305.65</v>
+      </c>
+      <c r="E152" s="23" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="F152" s="22" t="n">
+        <v>27353.1</v>
+      </c>
+      <c r="G152" s="22" t="n">
+        <v>27710.45</v>
+      </c>
+      <c r="H152" s="22" t="n">
+        <v>27298</v>
+      </c>
+      <c r="I152" s="22" t="n">
+        <v>27869.75</v>
+      </c>
+      <c r="J152" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K152" s="22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B153" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY MIDCAP 50</t>
+        </is>
+      </c>
+      <c r="C153" s="22" t="n">
+        <v>16520.35</v>
+      </c>
+      <c r="D153" s="22" t="n">
+        <v>-245.25</v>
+      </c>
+      <c r="E153" s="23" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="F153" s="22" t="n">
+        <v>16201.9</v>
+      </c>
+      <c r="G153" s="22" t="n">
+        <v>16705.65</v>
+      </c>
+      <c r="H153" s="22" t="n">
+        <v>16197.8</v>
+      </c>
+      <c r="I153" s="22" t="n">
+        <v>16765.6</v>
+      </c>
+      <c r="J153" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K153" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B154" s="22" t="inlineStr">
+        <is>
+          <t>INDIA VIX</t>
+        </is>
+      </c>
+      <c r="C154" s="22" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="D154" s="22" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E154" s="24" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="F154" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G154" s="22" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="H154" s="22" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="I154" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="J154" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B155" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY SMALLCAP 50</t>
+        </is>
+      </c>
+      <c r="C155" s="22" t="n">
+        <v>8167.25</v>
+      </c>
+      <c r="D155" s="22" t="n">
+        <v>-135.05</v>
+      </c>
+      <c r="E155" s="23" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="F155" s="22" t="n">
+        <v>7986.6</v>
+      </c>
+      <c r="G155" s="22" t="n">
+        <v>8260.6</v>
+      </c>
+      <c r="H155" s="22" t="n">
+        <v>7983.8</v>
+      </c>
+      <c r="I155" s="22" t="n">
+        <v>8302.299999999999</v>
+      </c>
+      <c r="J155" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K155" s="22" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B156" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY AUTO</t>
+        </is>
+      </c>
+      <c r="C156" s="22" t="n">
+        <v>27540.1</v>
+      </c>
+      <c r="D156" s="22" t="n">
+        <v>-618.75</v>
+      </c>
+      <c r="E156" s="23" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="F156" s="22" t="n">
+        <v>27196.4</v>
+      </c>
+      <c r="G156" s="22" t="n">
+        <v>27951.85</v>
+      </c>
+      <c r="H156" s="22" t="n">
+        <v>27133.55</v>
+      </c>
+      <c r="I156" s="22" t="n">
+        <v>28158.85</v>
+      </c>
+      <c r="J156" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K156" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B157" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FMCG</t>
+        </is>
+      </c>
+      <c r="C157" s="22" t="n">
+        <v>50751.65</v>
+      </c>
+      <c r="D157" s="22" t="n">
+        <v>-390.55</v>
+      </c>
+      <c r="E157" s="23" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="F157" s="22" t="n">
+        <v>49968.25</v>
+      </c>
+      <c r="G157" s="22" t="n">
+        <v>50879.5</v>
+      </c>
+      <c r="H157" s="22" t="n">
+        <v>49954.15</v>
+      </c>
+      <c r="I157" s="22" t="n">
+        <v>51142.2</v>
+      </c>
+      <c r="J157" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K157" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B158" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY IT</t>
+        </is>
+      </c>
+      <c r="C158" s="22" t="n">
+        <v>30272.95</v>
+      </c>
+      <c r="D158" s="22" t="n">
+        <v>-330.9</v>
+      </c>
+      <c r="E158" s="23" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="F158" s="22" t="n">
+        <v>30020.15</v>
+      </c>
+      <c r="G158" s="22" t="n">
+        <v>30587.3</v>
+      </c>
+      <c r="H158" s="22" t="n">
+        <v>29889.5</v>
+      </c>
+      <c r="I158" s="22" t="n">
+        <v>30603.85</v>
+      </c>
+      <c r="J158" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K158" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B159" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY METAL</t>
+        </is>
+      </c>
+      <c r="C159" s="22" t="n">
+        <v>12269.8</v>
+      </c>
+      <c r="D159" s="22" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="E159" s="24" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F159" s="22" t="n">
+        <v>11909.9</v>
+      </c>
+      <c r="G159" s="22" t="n">
+        <v>12344.8</v>
+      </c>
+      <c r="H159" s="22" t="n">
+        <v>11896</v>
+      </c>
+      <c r="I159" s="22" t="n">
+        <v>12240.65</v>
+      </c>
+      <c r="J159" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K159" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B160" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PHARMA</t>
+        </is>
+      </c>
+      <c r="C160" s="22" t="n">
+        <v>22956.7</v>
+      </c>
+      <c r="D160" s="22" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E160" s="24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F160" s="22" t="n">
+        <v>22385.3</v>
+      </c>
+      <c r="G160" s="22" t="n">
+        <v>22994.55</v>
+      </c>
+      <c r="H160" s="22" t="n">
+        <v>22354.1</v>
+      </c>
+      <c r="I160" s="22" t="n">
+        <v>22952.35</v>
+      </c>
+      <c r="J160" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K160" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B161" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PSU BANK</t>
+        </is>
+      </c>
+      <c r="C161" s="22" t="n">
+        <v>9639.35</v>
+      </c>
+      <c r="D161" s="22" t="n">
+        <v>-181.1</v>
+      </c>
+      <c r="E161" s="23" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="F161" s="22" t="n">
+        <v>9538.049999999999</v>
+      </c>
+      <c r="G161" s="22" t="n">
+        <v>9742.4</v>
+      </c>
+      <c r="H161" s="22" t="n">
+        <v>9526.5</v>
+      </c>
+      <c r="I161" s="22" t="n">
+        <v>9820.450000000001</v>
+      </c>
+      <c r="J161" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K161" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B162" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY REALTY</t>
+        </is>
+      </c>
+      <c r="C162" s="22" t="n">
+        <v>768.05</v>
+      </c>
+      <c r="D162" s="22" t="n">
+        <v>-12.55</v>
+      </c>
+      <c r="E162" s="23" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="F162" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="G162" s="22" t="n">
+        <v>770.65</v>
+      </c>
+      <c r="H162" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="I162" s="22" t="n">
+        <v>780.6</v>
+      </c>
+      <c r="J162" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K162" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B163" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY OIL &amp; GAS</t>
+        </is>
+      </c>
+      <c r="C163" s="22" t="n">
+        <v>12001.3</v>
+      </c>
+      <c r="D163" s="22" t="n">
+        <v>-263.6</v>
+      </c>
+      <c r="E163" s="23" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F163" s="22" t="n">
+        <v>12085.4</v>
+      </c>
+      <c r="G163" s="22" t="n">
+        <v>12159.55</v>
+      </c>
+      <c r="H163" s="22" t="n">
+        <v>11888.05</v>
+      </c>
+      <c r="I163" s="22" t="n">
+        <v>12264.9</v>
+      </c>
+      <c r="J163" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K163" s="22" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B164" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY100 LOW VOLATILITY 30</t>
+        </is>
+      </c>
+      <c r="C164" s="22" t="n">
+        <v>20280.2</v>
+      </c>
+      <c r="D164" s="22" t="n">
+        <v>-214.8</v>
+      </c>
+      <c r="E164" s="23" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="F164" s="22" t="n">
+        <v>20049.15</v>
+      </c>
+      <c r="G164" s="22" t="n">
+        <v>20326.65</v>
+      </c>
+      <c r="H164" s="22" t="n">
+        <v>20032.4</v>
+      </c>
+      <c r="I164" s="22" t="n">
+        <v>20495</v>
+      </c>
+      <c r="J164" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K164" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B165" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY200 MOMENTUM 30</t>
+        </is>
+      </c>
+      <c r="C165" s="22" t="n">
+        <v>30845.6</v>
+      </c>
+      <c r="D165" s="22" t="n">
+        <v>-515.35</v>
+      </c>
+      <c r="E165" s="23" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="F165" s="22" t="n">
+        <v>30408</v>
+      </c>
+      <c r="G165" s="22" t="n">
+        <v>31228.1</v>
+      </c>
+      <c r="H165" s="22" t="n">
+        <v>30395.65</v>
+      </c>
+      <c r="I165" s="22" t="n">
+        <v>31360.95</v>
+      </c>
+      <c r="J165" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K165" s="22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B166" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY HIGH BETA 50</t>
+        </is>
+      </c>
+      <c r="C166" s="22" t="n">
+        <v>3704.75</v>
+      </c>
+      <c r="D166" s="22" t="n">
+        <v>-76.84999999999999</v>
+      </c>
+      <c r="E166" s="23" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F166" s="22" t="n">
+        <v>3631.55</v>
+      </c>
+      <c r="G166" s="22" t="n">
+        <v>3751.85</v>
+      </c>
+      <c r="H166" s="22" t="n">
+        <v>3627.7</v>
+      </c>
+      <c r="I166" s="22" t="n">
+        <v>3781.6</v>
+      </c>
+      <c r="J166" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K166" s="22" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B167" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY COMMODITIES</t>
+        </is>
+      </c>
+      <c r="C167" s="22" t="n">
+        <v>9849.549999999999</v>
+      </c>
+      <c r="D167" s="22" t="n">
+        <v>-106.4</v>
+      </c>
+      <c r="E167" s="23" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="F167" s="22" t="n">
+        <v>9684.6</v>
+      </c>
+      <c r="G167" s="22" t="n">
+        <v>9892.25</v>
+      </c>
+      <c r="H167" s="22" t="n">
+        <v>9673.799999999999</v>
+      </c>
+      <c r="I167" s="22" t="n">
+        <v>9955.950000000001</v>
+      </c>
+      <c r="J167" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K167" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B168" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY ENERGY</t>
+        </is>
+      </c>
+      <c r="C168" s="22" t="n">
+        <v>36453.4</v>
+      </c>
+      <c r="D168" s="22" t="n">
+        <v>-591.8</v>
+      </c>
+      <c r="E168" s="23" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="F168" s="22" t="n">
+        <v>36014.35</v>
+      </c>
+      <c r="G168" s="22" t="n">
+        <v>36756.75</v>
+      </c>
+      <c r="H168" s="22" t="n">
+        <v>35972.7</v>
+      </c>
+      <c r="I168" s="22" t="n">
+        <v>37045.2</v>
+      </c>
+      <c r="J168" s="22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K168" s="22" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B169" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY INDIA DEFENCE</t>
+        </is>
+      </c>
+      <c r="C169" s="22" t="n">
+        <v>8166.5</v>
+      </c>
+      <c r="D169" s="22" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="E169" s="24" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F169" s="22" t="n">
+        <v>7936.05</v>
+      </c>
+      <c r="G169" s="22" t="n">
+        <v>8288.299999999999</v>
+      </c>
+      <c r="H169" s="22" t="n">
+        <v>7933.7</v>
+      </c>
+      <c r="I169" s="22" t="n">
+        <v>8126.8</v>
+      </c>
+      <c r="J169" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K169" s="22" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B170" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C170" s="22" t="n">
+        <v>24865.7</v>
+      </c>
+      <c r="D170" s="22" t="n">
+        <v>-312.95</v>
+      </c>
+      <c r="E170" s="23" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="F170" s="22" t="n">
+        <v>24659.25</v>
+      </c>
+      <c r="G170" s="22" t="n">
+        <v>24989.35</v>
+      </c>
+      <c r="H170" s="22" t="n">
+        <v>24603.5</v>
+      </c>
+      <c r="I170" s="22" t="n">
+        <v>25178.65</v>
+      </c>
+      <c r="J170" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K170" s="22" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B171" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY NEXT 50</t>
+        </is>
+      </c>
+      <c r="C171" s="22" t="n">
+        <v>68650.25</v>
+      </c>
+      <c r="D171" s="22" t="n">
+        <v>-1060.65</v>
+      </c>
+      <c r="E171" s="23" t="n">
+        <v>-1.52</v>
+      </c>
+      <c r="F171" s="22" t="n">
+        <v>67393.3</v>
+      </c>
+      <c r="G171" s="22" t="n">
+        <v>69144.45</v>
+      </c>
+      <c r="H171" s="22" t="n">
+        <v>67352.55</v>
+      </c>
+      <c r="I171" s="22" t="n">
+        <v>69710.89999999999</v>
+      </c>
+      <c r="J171" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K171" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B172" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY BANK</t>
+        </is>
+      </c>
+      <c r="C172" s="22" t="n">
+        <v>59839.65</v>
+      </c>
+      <c r="D172" s="22" t="n">
+        <v>-689.35</v>
+      </c>
+      <c r="E172" s="23" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="F172" s="22" t="n">
+        <v>59204.3</v>
+      </c>
+      <c r="G172" s="22" t="n">
+        <v>60177.5</v>
+      </c>
+      <c r="H172" s="22" t="n">
+        <v>59148</v>
+      </c>
+      <c r="I172" s="22" t="n">
+        <v>60529</v>
+      </c>
+      <c r="J172" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K172" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B173" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FINANCIAL SERVICES</t>
+        </is>
+      </c>
+      <c r="C173" s="22" t="n">
+        <v>27564.1</v>
+      </c>
+      <c r="D173" s="22" t="n">
+        <v>-305.65</v>
+      </c>
+      <c r="E173" s="23" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="F173" s="22" t="n">
+        <v>27353.1</v>
+      </c>
+      <c r="G173" s="22" t="n">
+        <v>27710.45</v>
+      </c>
+      <c r="H173" s="22" t="n">
+        <v>27298</v>
+      </c>
+      <c r="I173" s="22" t="n">
+        <v>27869.75</v>
+      </c>
+      <c r="J173" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K173" s="22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B174" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY MIDCAP 50</t>
+        </is>
+      </c>
+      <c r="C174" s="22" t="n">
+        <v>16520.35</v>
+      </c>
+      <c r="D174" s="22" t="n">
+        <v>-245.25</v>
+      </c>
+      <c r="E174" s="23" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="F174" s="22" t="n">
+        <v>16201.9</v>
+      </c>
+      <c r="G174" s="22" t="n">
+        <v>16705.65</v>
+      </c>
+      <c r="H174" s="22" t="n">
+        <v>16197.8</v>
+      </c>
+      <c r="I174" s="22" t="n">
+        <v>16765.6</v>
+      </c>
+      <c r="J174" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K174" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B175" s="22" t="inlineStr">
+        <is>
+          <t>INDIA VIX</t>
+        </is>
+      </c>
+      <c r="C175" s="22" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="D175" s="22" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E175" s="24" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="F175" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G175" s="22" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="H175" s="22" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="I175" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="J175" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B176" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY SMALLCAP 50</t>
+        </is>
+      </c>
+      <c r="C176" s="22" t="n">
+        <v>8167.25</v>
+      </c>
+      <c r="D176" s="22" t="n">
+        <v>-135.05</v>
+      </c>
+      <c r="E176" s="23" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="F176" s="22" t="n">
+        <v>7986.6</v>
+      </c>
+      <c r="G176" s="22" t="n">
+        <v>8260.6</v>
+      </c>
+      <c r="H176" s="22" t="n">
+        <v>7983.8</v>
+      </c>
+      <c r="I176" s="22" t="n">
+        <v>8302.299999999999</v>
+      </c>
+      <c r="J176" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K176" s="22" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B177" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY AUTO</t>
+        </is>
+      </c>
+      <c r="C177" s="22" t="n">
+        <v>27540.1</v>
+      </c>
+      <c r="D177" s="22" t="n">
+        <v>-618.75</v>
+      </c>
+      <c r="E177" s="23" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="F177" s="22" t="n">
+        <v>27196.4</v>
+      </c>
+      <c r="G177" s="22" t="n">
+        <v>27951.85</v>
+      </c>
+      <c r="H177" s="22" t="n">
+        <v>27133.55</v>
+      </c>
+      <c r="I177" s="22" t="n">
+        <v>28158.85</v>
+      </c>
+      <c r="J177" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K177" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B178" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FMCG</t>
+        </is>
+      </c>
+      <c r="C178" s="22" t="n">
+        <v>50751.65</v>
+      </c>
+      <c r="D178" s="22" t="n">
+        <v>-390.55</v>
+      </c>
+      <c r="E178" s="23" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="F178" s="22" t="n">
+        <v>49968.25</v>
+      </c>
+      <c r="G178" s="22" t="n">
+        <v>50879.5</v>
+      </c>
+      <c r="H178" s="22" t="n">
+        <v>49954.15</v>
+      </c>
+      <c r="I178" s="22" t="n">
+        <v>51142.2</v>
+      </c>
+      <c r="J178" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K178" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B179" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY IT</t>
+        </is>
+      </c>
+      <c r="C179" s="22" t="n">
+        <v>30272.95</v>
+      </c>
+      <c r="D179" s="22" t="n">
+        <v>-330.9</v>
+      </c>
+      <c r="E179" s="23" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="F179" s="22" t="n">
+        <v>30020.15</v>
+      </c>
+      <c r="G179" s="22" t="n">
+        <v>30587.3</v>
+      </c>
+      <c r="H179" s="22" t="n">
+        <v>29889.5</v>
+      </c>
+      <c r="I179" s="22" t="n">
+        <v>30603.85</v>
+      </c>
+      <c r="J179" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K179" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B180" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY METAL</t>
+        </is>
+      </c>
+      <c r="C180" s="22" t="n">
+        <v>12269.8</v>
+      </c>
+      <c r="D180" s="22" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="E180" s="24" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F180" s="22" t="n">
+        <v>11909.9</v>
+      </c>
+      <c r="G180" s="22" t="n">
+        <v>12344.8</v>
+      </c>
+      <c r="H180" s="22" t="n">
+        <v>11896</v>
+      </c>
+      <c r="I180" s="22" t="n">
+        <v>12240.65</v>
+      </c>
+      <c r="J180" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K180" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B181" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PHARMA</t>
+        </is>
+      </c>
+      <c r="C181" s="22" t="n">
+        <v>22956.7</v>
+      </c>
+      <c r="D181" s="22" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E181" s="24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F181" s="22" t="n">
+        <v>22385.3</v>
+      </c>
+      <c r="G181" s="22" t="n">
+        <v>22994.55</v>
+      </c>
+      <c r="H181" s="22" t="n">
+        <v>22354.1</v>
+      </c>
+      <c r="I181" s="22" t="n">
+        <v>22952.35</v>
+      </c>
+      <c r="J181" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K181" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B182" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PSU BANK</t>
+        </is>
+      </c>
+      <c r="C182" s="22" t="n">
+        <v>9639.35</v>
+      </c>
+      <c r="D182" s="22" t="n">
+        <v>-181.1</v>
+      </c>
+      <c r="E182" s="23" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="F182" s="22" t="n">
+        <v>9538.049999999999</v>
+      </c>
+      <c r="G182" s="22" t="n">
+        <v>9742.4</v>
+      </c>
+      <c r="H182" s="22" t="n">
+        <v>9526.5</v>
+      </c>
+      <c r="I182" s="22" t="n">
+        <v>9820.450000000001</v>
+      </c>
+      <c r="J182" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K182" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B183" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY REALTY</t>
+        </is>
+      </c>
+      <c r="C183" s="22" t="n">
+        <v>768.05</v>
+      </c>
+      <c r="D183" s="22" t="n">
+        <v>-12.55</v>
+      </c>
+      <c r="E183" s="23" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="F183" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="G183" s="22" t="n">
+        <v>770.65</v>
+      </c>
+      <c r="H183" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="I183" s="22" t="n">
+        <v>780.6</v>
+      </c>
+      <c r="J183" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K183" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B184" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY OIL &amp; GAS</t>
+        </is>
+      </c>
+      <c r="C184" s="22" t="n">
+        <v>12001.3</v>
+      </c>
+      <c r="D184" s="22" t="n">
+        <v>-263.6</v>
+      </c>
+      <c r="E184" s="23" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F184" s="22" t="n">
+        <v>12085.4</v>
+      </c>
+      <c r="G184" s="22" t="n">
+        <v>12159.55</v>
+      </c>
+      <c r="H184" s="22" t="n">
+        <v>11888.05</v>
+      </c>
+      <c r="I184" s="22" t="n">
+        <v>12264.9</v>
+      </c>
+      <c r="J184" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K184" s="22" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B185" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY100 LOW VOLATILITY 30</t>
+        </is>
+      </c>
+      <c r="C185" s="22" t="n">
+        <v>20280.2</v>
+      </c>
+      <c r="D185" s="22" t="n">
+        <v>-214.8</v>
+      </c>
+      <c r="E185" s="23" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="F185" s="22" t="n">
+        <v>20049.15</v>
+      </c>
+      <c r="G185" s="22" t="n">
+        <v>20326.65</v>
+      </c>
+      <c r="H185" s="22" t="n">
+        <v>20032.4</v>
+      </c>
+      <c r="I185" s="22" t="n">
+        <v>20495</v>
+      </c>
+      <c r="J185" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K185" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B186" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY200 MOMENTUM 30</t>
+        </is>
+      </c>
+      <c r="C186" s="22" t="n">
+        <v>30845.6</v>
+      </c>
+      <c r="D186" s="22" t="n">
+        <v>-515.35</v>
+      </c>
+      <c r="E186" s="23" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="F186" s="22" t="n">
+        <v>30408</v>
+      </c>
+      <c r="G186" s="22" t="n">
+        <v>31228.1</v>
+      </c>
+      <c r="H186" s="22" t="n">
+        <v>30395.65</v>
+      </c>
+      <c r="I186" s="22" t="n">
+        <v>31360.95</v>
+      </c>
+      <c r="J186" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K186" s="22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B187" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY HIGH BETA 50</t>
+        </is>
+      </c>
+      <c r="C187" s="22" t="n">
+        <v>3704.75</v>
+      </c>
+      <c r="D187" s="22" t="n">
+        <v>-76.84999999999999</v>
+      </c>
+      <c r="E187" s="23" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F187" s="22" t="n">
+        <v>3631.55</v>
+      </c>
+      <c r="G187" s="22" t="n">
+        <v>3751.85</v>
+      </c>
+      <c r="H187" s="22" t="n">
+        <v>3627.7</v>
+      </c>
+      <c r="I187" s="22" t="n">
+        <v>3781.6</v>
+      </c>
+      <c r="J187" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K187" s="22" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B188" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY COMMODITIES</t>
+        </is>
+      </c>
+      <c r="C188" s="22" t="n">
+        <v>9849.549999999999</v>
+      </c>
+      <c r="D188" s="22" t="n">
+        <v>-106.4</v>
+      </c>
+      <c r="E188" s="23" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="F188" s="22" t="n">
+        <v>9684.6</v>
+      </c>
+      <c r="G188" s="22" t="n">
+        <v>9892.25</v>
+      </c>
+      <c r="H188" s="22" t="n">
+        <v>9673.799999999999</v>
+      </c>
+      <c r="I188" s="22" t="n">
+        <v>9955.950000000001</v>
+      </c>
+      <c r="J188" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K188" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B189" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY ENERGY</t>
+        </is>
+      </c>
+      <c r="C189" s="22" t="n">
+        <v>36453.4</v>
+      </c>
+      <c r="D189" s="22" t="n">
+        <v>-591.8</v>
+      </c>
+      <c r="E189" s="23" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="F189" s="22" t="n">
+        <v>36014.35</v>
+      </c>
+      <c r="G189" s="22" t="n">
+        <v>36756.75</v>
+      </c>
+      <c r="H189" s="22" t="n">
+        <v>35972.7</v>
+      </c>
+      <c r="I189" s="22" t="n">
+        <v>37045.2</v>
+      </c>
+      <c r="J189" s="22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K189" s="22" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B190" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY INDIA DEFENCE</t>
+        </is>
+      </c>
+      <c r="C190" s="22" t="n">
+        <v>8166.5</v>
+      </c>
+      <c r="D190" s="22" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="E190" s="24" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F190" s="22" t="n">
+        <v>7936.05</v>
+      </c>
+      <c r="G190" s="22" t="n">
+        <v>8288.299999999999</v>
+      </c>
+      <c r="H190" s="22" t="n">
+        <v>7933.7</v>
+      </c>
+      <c r="I190" s="22" t="n">
+        <v>8126.8</v>
+      </c>
+      <c r="J190" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K190" s="22" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B191" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C191" s="22" t="n">
+        <v>24865.7</v>
+      </c>
+      <c r="D191" s="22" t="n">
+        <v>-312.95</v>
+      </c>
+      <c r="E191" s="23" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="F191" s="22" t="n">
+        <v>24659.25</v>
+      </c>
+      <c r="G191" s="22" t="n">
+        <v>24989.35</v>
+      </c>
+      <c r="H191" s="22" t="n">
+        <v>24603.5</v>
+      </c>
+      <c r="I191" s="22" t="n">
+        <v>25178.65</v>
+      </c>
+      <c r="J191" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K191" s="22" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B192" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY NEXT 50</t>
+        </is>
+      </c>
+      <c r="C192" s="22" t="n">
+        <v>68650.25</v>
+      </c>
+      <c r="D192" s="22" t="n">
+        <v>-1060.65</v>
+      </c>
+      <c r="E192" s="23" t="n">
+        <v>-1.52</v>
+      </c>
+      <c r="F192" s="22" t="n">
+        <v>67393.3</v>
+      </c>
+      <c r="G192" s="22" t="n">
+        <v>69144.45</v>
+      </c>
+      <c r="H192" s="22" t="n">
+        <v>67352.55</v>
+      </c>
+      <c r="I192" s="22" t="n">
+        <v>69710.89999999999</v>
+      </c>
+      <c r="J192" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K192" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B193" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY BANK</t>
+        </is>
+      </c>
+      <c r="C193" s="22" t="n">
+        <v>59839.65</v>
+      </c>
+      <c r="D193" s="22" t="n">
+        <v>-689.35</v>
+      </c>
+      <c r="E193" s="23" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="F193" s="22" t="n">
+        <v>59204.3</v>
+      </c>
+      <c r="G193" s="22" t="n">
+        <v>60177.5</v>
+      </c>
+      <c r="H193" s="22" t="n">
+        <v>59148</v>
+      </c>
+      <c r="I193" s="22" t="n">
+        <v>60529</v>
+      </c>
+      <c r="J193" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K193" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B194" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FINANCIAL SERVICES</t>
+        </is>
+      </c>
+      <c r="C194" s="22" t="n">
+        <v>27564.1</v>
+      </c>
+      <c r="D194" s="22" t="n">
+        <v>-305.65</v>
+      </c>
+      <c r="E194" s="23" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="F194" s="22" t="n">
+        <v>27353.1</v>
+      </c>
+      <c r="G194" s="22" t="n">
+        <v>27710.45</v>
+      </c>
+      <c r="H194" s="22" t="n">
+        <v>27298</v>
+      </c>
+      <c r="I194" s="22" t="n">
+        <v>27869.75</v>
+      </c>
+      <c r="J194" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K194" s="22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B195" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY MIDCAP 50</t>
+        </is>
+      </c>
+      <c r="C195" s="22" t="n">
+        <v>16520.35</v>
+      </c>
+      <c r="D195" s="22" t="n">
+        <v>-245.25</v>
+      </c>
+      <c r="E195" s="23" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="F195" s="22" t="n">
+        <v>16201.9</v>
+      </c>
+      <c r="G195" s="22" t="n">
+        <v>16705.65</v>
+      </c>
+      <c r="H195" s="22" t="n">
+        <v>16197.8</v>
+      </c>
+      <c r="I195" s="22" t="n">
+        <v>16765.6</v>
+      </c>
+      <c r="J195" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K195" s="22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B196" s="22" t="inlineStr">
+        <is>
+          <t>INDIA VIX</t>
+        </is>
+      </c>
+      <c r="C196" s="22" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="D196" s="22" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E196" s="24" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="F196" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G196" s="22" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="H196" s="22" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="I196" s="22" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="J196" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K196" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B197" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY SMALLCAP 50</t>
+        </is>
+      </c>
+      <c r="C197" s="22" t="n">
+        <v>8167.25</v>
+      </c>
+      <c r="D197" s="22" t="n">
+        <v>-135.05</v>
+      </c>
+      <c r="E197" s="23" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="F197" s="22" t="n">
+        <v>7986.6</v>
+      </c>
+      <c r="G197" s="22" t="n">
+        <v>8260.6</v>
+      </c>
+      <c r="H197" s="22" t="n">
+        <v>7983.8</v>
+      </c>
+      <c r="I197" s="22" t="n">
+        <v>8302.299999999999</v>
+      </c>
+      <c r="J197" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K197" s="22" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B198" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY AUTO</t>
+        </is>
+      </c>
+      <c r="C198" s="22" t="n">
+        <v>27540.1</v>
+      </c>
+      <c r="D198" s="22" t="n">
+        <v>-618.75</v>
+      </c>
+      <c r="E198" s="23" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="F198" s="22" t="n">
+        <v>27196.4</v>
+      </c>
+      <c r="G198" s="22" t="n">
+        <v>27951.85</v>
+      </c>
+      <c r="H198" s="22" t="n">
+        <v>27133.55</v>
+      </c>
+      <c r="I198" s="22" t="n">
+        <v>28158.85</v>
+      </c>
+      <c r="J198" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K198" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B199" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY FMCG</t>
+        </is>
+      </c>
+      <c r="C199" s="22" t="n">
+        <v>50751.65</v>
+      </c>
+      <c r="D199" s="22" t="n">
+        <v>-390.55</v>
+      </c>
+      <c r="E199" s="23" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="F199" s="22" t="n">
+        <v>49968.25</v>
+      </c>
+      <c r="G199" s="22" t="n">
+        <v>50879.5</v>
+      </c>
+      <c r="H199" s="22" t="n">
+        <v>49954.15</v>
+      </c>
+      <c r="I199" s="22" t="n">
+        <v>51142.2</v>
+      </c>
+      <c r="J199" s="22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K199" s="22" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B200" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY IT</t>
+        </is>
+      </c>
+      <c r="C200" s="22" t="n">
+        <v>30272.95</v>
+      </c>
+      <c r="D200" s="22" t="n">
+        <v>-330.9</v>
+      </c>
+      <c r="E200" s="23" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="F200" s="22" t="n">
+        <v>30020.15</v>
+      </c>
+      <c r="G200" s="22" t="n">
+        <v>30587.3</v>
+      </c>
+      <c r="H200" s="22" t="n">
+        <v>29889.5</v>
+      </c>
+      <c r="I200" s="22" t="n">
+        <v>30603.85</v>
+      </c>
+      <c r="J200" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K200" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B201" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY METAL</t>
+        </is>
+      </c>
+      <c r="C201" s="22" t="n">
+        <v>12269.8</v>
+      </c>
+      <c r="D201" s="22" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="E201" s="24" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F201" s="22" t="n">
+        <v>11909.9</v>
+      </c>
+      <c r="G201" s="22" t="n">
+        <v>12344.8</v>
+      </c>
+      <c r="H201" s="22" t="n">
+        <v>11896</v>
+      </c>
+      <c r="I201" s="22" t="n">
+        <v>12240.65</v>
+      </c>
+      <c r="J201" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K201" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B202" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PHARMA</t>
+        </is>
+      </c>
+      <c r="C202" s="22" t="n">
+        <v>22956.7</v>
+      </c>
+      <c r="D202" s="22" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E202" s="24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F202" s="22" t="n">
+        <v>22385.3</v>
+      </c>
+      <c r="G202" s="22" t="n">
+        <v>22994.55</v>
+      </c>
+      <c r="H202" s="22" t="n">
+        <v>22354.1</v>
+      </c>
+      <c r="I202" s="22" t="n">
+        <v>22952.35</v>
+      </c>
+      <c r="J202" s="22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K202" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B203" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PSU BANK</t>
+        </is>
+      </c>
+      <c r="C203" s="22" t="n">
+        <v>9639.35</v>
+      </c>
+      <c r="D203" s="22" t="n">
+        <v>-181.1</v>
+      </c>
+      <c r="E203" s="23" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="F203" s="22" t="n">
+        <v>9538.049999999999</v>
+      </c>
+      <c r="G203" s="22" t="n">
+        <v>9742.4</v>
+      </c>
+      <c r="H203" s="22" t="n">
+        <v>9526.5</v>
+      </c>
+      <c r="I203" s="22" t="n">
+        <v>9820.450000000001</v>
+      </c>
+      <c r="J203" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K203" s="22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B204" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY REALTY</t>
+        </is>
+      </c>
+      <c r="C204" s="22" t="n">
+        <v>768.05</v>
+      </c>
+      <c r="D204" s="22" t="n">
+        <v>-12.55</v>
+      </c>
+      <c r="E204" s="23" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="F204" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="G204" s="22" t="n">
+        <v>770.65</v>
+      </c>
+      <c r="H204" s="22" t="n">
+        <v>751.75</v>
+      </c>
+      <c r="I204" s="22" t="n">
+        <v>780.6</v>
+      </c>
+      <c r="J204" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K204" s="22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B205" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY OIL &amp; GAS</t>
+        </is>
+      </c>
+      <c r="C205" s="22" t="n">
+        <v>12001.3</v>
+      </c>
+      <c r="D205" s="22" t="n">
+        <v>-263.6</v>
+      </c>
+      <c r="E205" s="23" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F205" s="22" t="n">
+        <v>12085.4</v>
+      </c>
+      <c r="G205" s="22" t="n">
+        <v>12159.55</v>
+      </c>
+      <c r="H205" s="22" t="n">
+        <v>11888.05</v>
+      </c>
+      <c r="I205" s="22" t="n">
+        <v>12264.9</v>
+      </c>
+      <c r="J205" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K205" s="22" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B206" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY100 LOW VOLATILITY 30</t>
+        </is>
+      </c>
+      <c r="C206" s="22" t="n">
+        <v>20280.2</v>
+      </c>
+      <c r="D206" s="22" t="n">
+        <v>-214.8</v>
+      </c>
+      <c r="E206" s="23" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="F206" s="22" t="n">
+        <v>20049.15</v>
+      </c>
+      <c r="G206" s="22" t="n">
+        <v>20326.65</v>
+      </c>
+      <c r="H206" s="22" t="n">
+        <v>20032.4</v>
+      </c>
+      <c r="I206" s="22" t="n">
+        <v>20495</v>
+      </c>
+      <c r="J206" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K206" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B207" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY200 MOMENTUM 30</t>
+        </is>
+      </c>
+      <c r="C207" s="22" t="n">
+        <v>30845.6</v>
+      </c>
+      <c r="D207" s="22" t="n">
+        <v>-515.35</v>
+      </c>
+      <c r="E207" s="23" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="F207" s="22" t="n">
+        <v>30408</v>
+      </c>
+      <c r="G207" s="22" t="n">
+        <v>31228.1</v>
+      </c>
+      <c r="H207" s="22" t="n">
+        <v>30395.65</v>
+      </c>
+      <c r="I207" s="22" t="n">
+        <v>31360.95</v>
+      </c>
+      <c r="J207" s="22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K207" s="22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B208" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY HIGH BETA 50</t>
+        </is>
+      </c>
+      <c r="C208" s="22" t="n">
+        <v>3704.75</v>
+      </c>
+      <c r="D208" s="22" t="n">
+        <v>-76.84999999999999</v>
+      </c>
+      <c r="E208" s="23" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F208" s="22" t="n">
+        <v>3631.55</v>
+      </c>
+      <c r="G208" s="22" t="n">
+        <v>3751.85</v>
+      </c>
+      <c r="H208" s="22" t="n">
+        <v>3627.7</v>
+      </c>
+      <c r="I208" s="22" t="n">
+        <v>3781.6</v>
+      </c>
+      <c r="J208" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K208" s="22" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B209" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY COMMODITIES</t>
+        </is>
+      </c>
+      <c r="C209" s="22" t="n">
+        <v>9849.549999999999</v>
+      </c>
+      <c r="D209" s="22" t="n">
+        <v>-106.4</v>
+      </c>
+      <c r="E209" s="23" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="F209" s="22" t="n">
+        <v>9684.6</v>
+      </c>
+      <c r="G209" s="22" t="n">
+        <v>9892.25</v>
+      </c>
+      <c r="H209" s="22" t="n">
+        <v>9673.799999999999</v>
+      </c>
+      <c r="I209" s="22" t="n">
+        <v>9955.950000000001</v>
+      </c>
+      <c r="J209" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K209" s="22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B210" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY ENERGY</t>
+        </is>
+      </c>
+      <c r="C210" s="22" t="n">
+        <v>36453.4</v>
+      </c>
+      <c r="D210" s="22" t="n">
+        <v>-591.8</v>
+      </c>
+      <c r="E210" s="23" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="F210" s="22" t="n">
+        <v>36014.35</v>
+      </c>
+      <c r="G210" s="22" t="n">
+        <v>36756.75</v>
+      </c>
+      <c r="H210" s="22" t="n">
+        <v>35972.7</v>
+      </c>
+      <c r="I210" s="22" t="n">
+        <v>37045.2</v>
+      </c>
+      <c r="J210" s="22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K210" s="22" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B211" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY INDIA DEFENCE</t>
+        </is>
+      </c>
+      <c r="C211" s="22" t="n">
+        <v>8166.5</v>
+      </c>
+      <c r="D211" s="22" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="E211" s="24" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F211" s="22" t="n">
+        <v>7936.05</v>
+      </c>
+      <c r="G211" s="22" t="n">
+        <v>8288.299999999999</v>
+      </c>
+      <c r="H211" s="22" t="n">
+        <v>7933.7</v>
+      </c>
+      <c r="I211" s="22" t="n">
+        <v>8126.8</v>
+      </c>
+      <c r="J211" s="22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K211" s="22" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -7820,7 +10646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15.44140625" bestFit="1" customWidth="1" style="18" min="1" max="1"/>
@@ -8454,6 +11280,330 @@
         <v>1029.99</v>
       </c>
       <c r="G23" s="22" t="n">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>TATAGOLD</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>0.8100000000000005</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>5.259740259740263</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G24" s="22" t="n">
+        <v>7.14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>TATSILV</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>8.771929824561404</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>8.56</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>GOLDBEES</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>138.54</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>6.939999999999998</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>5.273556231003038</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="G26" s="22" t="n">
+        <v>65.84999999999999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>LIQUIDBEES</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>0.009999999999990905</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>0.001000010000099091</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>1029.99</v>
+      </c>
+      <c r="G27" s="22" t="n">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>TATAGOLD</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <v>0.8100000000000005</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <v>5.259740259740263</v>
+      </c>
+      <c r="F28" s="22" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G28" s="22" t="n">
+        <v>7.14</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>TATSILV</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>8.771929824561404</v>
+      </c>
+      <c r="F29" s="22" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="G29" s="22" t="n">
+        <v>8.56</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>GOLDBEES</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>138.54</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <v>6.939999999999998</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <v>5.273556231003038</v>
+      </c>
+      <c r="F30" s="22" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="G30" s="22" t="n">
+        <v>65.84999999999999</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>LIQUIDBEES</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <v>0.009999999999990905</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <v>0.001000010000099091</v>
+      </c>
+      <c r="F31" s="22" t="n">
+        <v>1029.99</v>
+      </c>
+      <c r="G31" s="22" t="n">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>TATAGOLD</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="D32" s="22" t="n">
+        <v>0.8100000000000005</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>5.259740259740263</v>
+      </c>
+      <c r="F32" s="22" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G32" s="22" t="n">
+        <v>7.14</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>TATSILV</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D33" s="22" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <v>8.771929824561404</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <v>8.56</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>GOLDBEES</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n">
+        <v>138.54</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <v>6.939999999999998</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <v>5.273556231003038</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>65.84999999999999</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>LIQUIDBEES</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D35" s="22" t="n">
+        <v>0.009999999999990905</v>
+      </c>
+      <c r="E35" s="22" t="n">
+        <v>0.001000010000099091</v>
+      </c>
+      <c r="F35" s="22" t="n">
+        <v>1029.99</v>
+      </c>
+      <c r="G35" s="22" t="n">
         <v>970</v>
       </c>
     </row>
@@ -8468,7 +11618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" ht="27.6" customHeight="1" s="18">
@@ -8618,6 +11768,78 @@
         <v>156.3437</v>
       </c>
       <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>91.2092</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>0.8485</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>0.7439</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>156.3437</v>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>91.2092</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>0.8485</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>0.7439</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>156.3437</v>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>91.2092</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>0.8485</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.7439</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>156.3437</v>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
@@ -8634,7 +11856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" ht="27.6" customHeight="1" s="18">
@@ -9514,6 +12736,672 @@
         </is>
       </c>
       <c r="I22" s="22" t="n">
+        <v>-4.48</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>24865.7</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="I23" s="22" t="n">
+        <v>-6.09</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY BANK</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>59839.65</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>-2.39</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY IT</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>30272.95</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>COFORGE</t>
+        </is>
+      </c>
+      <c r="I25" s="22" t="n">
+        <v>-1.59</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY AUTO</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>27540.1</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>TIINDIA</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>-3.51</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PHARMA</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>22956.7</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>WOCKPHARMA</t>
+        </is>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>-3.66</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY METAL</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>12269.8</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PSU BANK</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>9639.35</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>MAHABANK</t>
+        </is>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>-3.48</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY INDIA DEFENCE</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>8166.5</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>-2.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:06</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY OIL &amp; GAS</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
+        <v>12001.3</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>-4.48</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY 50</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n">
+        <v>24865.7</v>
+      </c>
+      <c r="D32" s="22" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>-6.09</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY BANK</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>59839.65</v>
+      </c>
+      <c r="D33" s="22" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="G33" s="22" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>-2.39</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY IT</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n">
+        <v>30272.95</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" s="22" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>COFORGE</t>
+        </is>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>-1.59</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY AUTO</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="n">
+        <v>27540.1</v>
+      </c>
+      <c r="D35" s="22" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="E35" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F35" s="22" t="inlineStr">
+        <is>
+          <t>TIINDIA</t>
+        </is>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="H35" s="22" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>-3.51</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PHARMA</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="n">
+        <v>22956.7</v>
+      </c>
+      <c r="D36" s="22" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E36" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="F36" s="22" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="G36" s="22" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t>WOCKPHARMA</t>
+        </is>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>-3.66</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY METAL</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="n">
+        <v>12269.8</v>
+      </c>
+      <c r="D37" s="22" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E37" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="G37" s="22" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="H37" s="22" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY PSU BANK</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="n">
+        <v>9639.35</v>
+      </c>
+      <c r="D38" s="22" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F38" s="22" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="G38" s="22" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="H38" s="22" t="inlineStr">
+        <is>
+          <t>MAHABANK</t>
+        </is>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>-3.48</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY INDIA DEFENCE</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="n">
+        <v>8166.5</v>
+      </c>
+      <c r="D39" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>-2.6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:07</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>NIFTY OIL &amp; GAS</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="n">
+        <v>12001.3</v>
+      </c>
+      <c r="D40" s="22" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="E40" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="I40" s="22" t="n">
         <v>-4.48</v>
       </c>
     </row>

</xml_diff>